<commit_message>
Actualizacion de datos financieros en Excel
</commit_message>
<xml_diff>
--- a/Datos/Gestion Proyecto Fatima.xlsx
+++ b/Datos/Gestion Proyecto Fatima.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP I5\Documents\Dashboard_Obras\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8599A9C1-59E8-4887-B75A-04A85309248A}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003631C2-CA49-4C65-8485-504752E6D679}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="755" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="763" uniqueCount="345">
   <si>
     <t>PRESUPUESTO TOTAL</t>
   </si>
@@ -1045,6 +1045,24 @@
   </si>
   <si>
     <t>Fatima</t>
+  </si>
+  <si>
+    <t>Centro</t>
+  </si>
+  <si>
+    <t>Izp</t>
+  </si>
+  <si>
+    <t>General</t>
+  </si>
+  <si>
+    <t>Hospital</t>
+  </si>
+  <si>
+    <t>Estadio</t>
+  </si>
+  <si>
+    <t>Graderia</t>
   </si>
 </sst>
 </file>
@@ -1495,13 +1513,13 @@
     <xf numFmtId="164" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -5391,7 +5409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FB8E136-486C-4EB9-920D-6287CDC3043B}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.42578125" style="32"/>
@@ -5474,16 +5492,345 @@
         <v>11419.96</v>
       </c>
       <c r="I2" s="72">
-        <f t="shared" ref="I2:J2" si="0">C2/$B$2</f>
+        <f>C2/B2</f>
         <v>0.49710716525496096</v>
       </c>
       <c r="J2" s="72">
-        <f t="shared" si="0"/>
+        <f>D2/B2</f>
         <v>0.75770847201117075</v>
       </c>
       <c r="K2" s="68">
         <f>B2-C2</f>
         <v>22037.563618134853</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="71" t="s">
+        <v>339</v>
+      </c>
+      <c r="B3" s="68">
+        <v>10000</v>
+      </c>
+      <c r="C3" s="69">
+        <v>2000</v>
+      </c>
+      <c r="D3" s="68">
+        <v>5000</v>
+      </c>
+      <c r="E3" s="68">
+        <v>21785.03</v>
+      </c>
+      <c r="F3" s="68">
+        <f t="shared" ref="F3:F10" si="0">C3-D3</f>
+        <v>-3000</v>
+      </c>
+      <c r="G3" s="68">
+        <f t="shared" ref="G3:G10" si="1">C3-E3</f>
+        <v>-19785.03</v>
+      </c>
+      <c r="H3" s="68">
+        <f t="shared" ref="H3:H10" si="2">D3-E3</f>
+        <v>-16785.03</v>
+      </c>
+      <c r="I3" s="72">
+        <f t="shared" ref="I3:I10" si="3">C3/B3</f>
+        <v>0.2</v>
+      </c>
+      <c r="J3" s="72">
+        <f t="shared" ref="J3:J10" si="4">D3/B3</f>
+        <v>0.5</v>
+      </c>
+      <c r="K3" s="68">
+        <f t="shared" ref="K3:K10" si="5">B3-C3</f>
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="71" t="s">
+        <v>340</v>
+      </c>
+      <c r="B4" s="68">
+        <v>50000</v>
+      </c>
+      <c r="C4" s="69">
+        <v>25000</v>
+      </c>
+      <c r="D4" s="68">
+        <v>28000</v>
+      </c>
+      <c r="E4" s="68">
+        <v>21786.03</v>
+      </c>
+      <c r="F4" s="68">
+        <f t="shared" si="0"/>
+        <v>-3000</v>
+      </c>
+      <c r="G4" s="68">
+        <f t="shared" si="1"/>
+        <v>3213.9700000000012</v>
+      </c>
+      <c r="H4" s="68">
+        <f t="shared" si="2"/>
+        <v>6213.9700000000012</v>
+      </c>
+      <c r="I4" s="72">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="J4" s="72">
+        <f t="shared" si="4"/>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="K4" s="68">
+        <f t="shared" si="5"/>
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="71" t="s">
+        <v>341</v>
+      </c>
+      <c r="B5" s="68">
+        <v>25000</v>
+      </c>
+      <c r="C5" s="69">
+        <f>Dashboard!C17</f>
+        <v>17239.126381865146</v>
+      </c>
+      <c r="D5" s="68">
+        <v>20000</v>
+      </c>
+      <c r="E5" s="68">
+        <v>21787.03</v>
+      </c>
+      <c r="F5" s="68">
+        <f t="shared" si="0"/>
+        <v>-2760.873618134854</v>
+      </c>
+      <c r="G5" s="68">
+        <f t="shared" si="1"/>
+        <v>-4547.9036181348529</v>
+      </c>
+      <c r="H5" s="68">
+        <f t="shared" si="2"/>
+        <v>-1787.0299999999988</v>
+      </c>
+      <c r="I5" s="72">
+        <f t="shared" si="3"/>
+        <v>0.68956505527460588</v>
+      </c>
+      <c r="J5" s="72">
+        <f t="shared" si="4"/>
+        <v>0.8</v>
+      </c>
+      <c r="K5" s="68">
+        <f t="shared" si="5"/>
+        <v>7760.873618134854</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="71" t="s">
+        <v>342</v>
+      </c>
+      <c r="B6" s="68">
+        <v>50000</v>
+      </c>
+      <c r="C6" s="69">
+        <v>23000</v>
+      </c>
+      <c r="D6" s="68">
+        <v>30000</v>
+      </c>
+      <c r="E6" s="68">
+        <v>21788.03</v>
+      </c>
+      <c r="F6" s="68">
+        <f t="shared" si="0"/>
+        <v>-7000</v>
+      </c>
+      <c r="G6" s="68">
+        <f t="shared" si="1"/>
+        <v>1211.9700000000012</v>
+      </c>
+      <c r="H6" s="68">
+        <f t="shared" si="2"/>
+        <v>8211.9700000000012</v>
+      </c>
+      <c r="I6" s="72">
+        <f t="shared" si="3"/>
+        <v>0.46</v>
+      </c>
+      <c r="J6" s="72">
+        <f t="shared" si="4"/>
+        <v>0.6</v>
+      </c>
+      <c r="K6" s="68">
+        <f t="shared" si="5"/>
+        <v>27000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="71" t="s">
+        <v>343</v>
+      </c>
+      <c r="B7" s="68">
+        <v>60000</v>
+      </c>
+      <c r="C7" s="69">
+        <v>12000</v>
+      </c>
+      <c r="D7" s="68">
+        <v>30000</v>
+      </c>
+      <c r="E7" s="68">
+        <v>21789.03</v>
+      </c>
+      <c r="F7" s="68">
+        <f t="shared" si="0"/>
+        <v>-18000</v>
+      </c>
+      <c r="G7" s="68">
+        <f t="shared" si="1"/>
+        <v>-9789.0299999999988</v>
+      </c>
+      <c r="H7" s="68">
+        <f t="shared" si="2"/>
+        <v>8210.9700000000012</v>
+      </c>
+      <c r="I7" s="72">
+        <f t="shared" si="3"/>
+        <v>0.2</v>
+      </c>
+      <c r="J7" s="72">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="K7" s="68">
+        <f t="shared" si="5"/>
+        <v>48000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="71" t="s">
+        <v>344</v>
+      </c>
+      <c r="B8" s="68">
+        <v>70000</v>
+      </c>
+      <c r="C8" s="69">
+        <v>35000</v>
+      </c>
+      <c r="D8" s="68">
+        <v>35000</v>
+      </c>
+      <c r="E8" s="68">
+        <v>21790.03</v>
+      </c>
+      <c r="F8" s="68">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="68">
+        <f t="shared" si="1"/>
+        <v>13209.970000000001</v>
+      </c>
+      <c r="H8" s="68">
+        <f t="shared" si="2"/>
+        <v>13209.970000000001</v>
+      </c>
+      <c r="I8" s="72">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="J8" s="72">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="K8" s="68">
+        <f t="shared" si="5"/>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="71" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="68">
+        <v>60000</v>
+      </c>
+      <c r="C9" s="69">
+        <v>25000</v>
+      </c>
+      <c r="D9" s="68">
+        <v>30000</v>
+      </c>
+      <c r="E9" s="68">
+        <v>21791.03</v>
+      </c>
+      <c r="F9" s="68">
+        <f t="shared" si="0"/>
+        <v>-5000</v>
+      </c>
+      <c r="G9" s="68">
+        <f t="shared" si="1"/>
+        <v>3208.9700000000012</v>
+      </c>
+      <c r="H9" s="68">
+        <f t="shared" si="2"/>
+        <v>8208.9700000000012</v>
+      </c>
+      <c r="I9" s="72">
+        <f t="shared" si="3"/>
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="J9" s="72">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="K9" s="68">
+        <f t="shared" si="5"/>
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="71" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" s="68">
+        <v>45000</v>
+      </c>
+      <c r="C10" s="69">
+        <v>20000</v>
+      </c>
+      <c r="D10" s="68">
+        <v>20000</v>
+      </c>
+      <c r="E10" s="68">
+        <v>21792.03</v>
+      </c>
+      <c r="F10" s="68">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G10" s="68">
+        <f t="shared" si="1"/>
+        <v>-1792.0299999999988</v>
+      </c>
+      <c r="H10" s="68">
+        <f t="shared" si="2"/>
+        <v>-1792.0299999999988</v>
+      </c>
+      <c r="I10" s="72">
+        <f t="shared" si="3"/>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="J10" s="72">
+        <f t="shared" si="4"/>
+        <v>0.44444444444444442</v>
+      </c>
+      <c r="K10" s="68">
+        <f t="shared" si="5"/>
+        <v>25000</v>
       </c>
     </row>
   </sheetData>
@@ -5507,28 +5854,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="76" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="73" t="s">
@@ -5564,7 +5911,7 @@
         <v>22037.563618134853</v>
       </c>
       <c r="F5" s="74"/>
-      <c r="G5" s="76">
+      <c r="G5" s="78">
         <f>C5/A5</f>
         <v>0.49710716525496096</v>
       </c>
@@ -5614,7 +5961,7 @@
         <v>11419.963618134854</v>
       </c>
       <c r="F8" s="74"/>
-      <c r="G8" s="76">
+      <c r="G8" s="78">
         <f>C8/A8</f>
         <v>0.65606652639833785</v>
       </c>
@@ -5848,6 +6195,14 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A8:B9"/>
+    <mergeCell ref="C8:D9"/>
+    <mergeCell ref="E8:F9"/>
+    <mergeCell ref="G8:H9"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="E4:F4"/>
@@ -5857,14 +6212,6 @@
     <mergeCell ref="E5:F6"/>
     <mergeCell ref="G5:H6"/>
     <mergeCell ref="C4:D4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="A8:B9"/>
-    <mergeCell ref="C8:D9"/>
-    <mergeCell ref="E8:F9"/>
-    <mergeCell ref="G8:H9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5884,20 +6231,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -6039,32 +6386,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="76" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
+      <c r="B1" s="77"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
@@ -10512,38 +10859,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" s="77" t="s">
+      <c r="A1" s="76" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="77"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
-      <c r="H1" s="78"/>
-      <c r="I1" s="78"/>
-      <c r="J1" s="78"/>
-      <c r="K1" s="78"/>
-      <c r="L1" s="78"/>
-      <c r="M1" s="78"/>
-      <c r="N1" s="78"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="77"/>
+      <c r="D1" s="77"/>
+      <c r="E1" s="77"/>
+      <c r="F1" s="77"/>
+      <c r="G1" s="77"/>
+      <c r="H1" s="77"/>
+      <c r="I1" s="77"/>
+      <c r="J1" s="77"/>
+      <c r="K1" s="77"/>
+      <c r="L1" s="77"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A2" s="78"/>
-      <c r="B2" s="78"/>
-      <c r="C2" s="78"/>
-      <c r="D2" s="78"/>
-      <c r="E2" s="78"/>
-      <c r="F2" s="78"/>
-      <c r="G2" s="78"/>
-      <c r="H2" s="78"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="78"/>
-      <c r="L2" s="78"/>
-      <c r="M2" s="78"/>
-      <c r="N2" s="78"/>
+      <c r="A2" s="77"/>
+      <c r="B2" s="77"/>
+      <c r="C2" s="77"/>
+      <c r="D2" s="77"/>
+      <c r="E2" s="77"/>
+      <c r="F2" s="77"/>
+      <c r="G2" s="77"/>
+      <c r="H2" s="77"/>
+      <c r="I2" s="77"/>
+      <c r="J2" s="77"/>
+      <c r="K2" s="77"/>
+      <c r="L2" s="77"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="77"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">

</xml_diff>